<commit_message>
Adjusted data cleaning code to fix problem with cities with enyes.
</commit_message>
<xml_diff>
--- a/data/clean/births_clean.xlsx
+++ b/data/clean/births_clean.xlsx
@@ -893,7 +893,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>BANGUED (CAPITAL)</t>
+          <t>BANGUED</t>
         </is>
       </c>
       <c r="B19" t="n">
@@ -1643,7 +1643,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>KABUGAO (CAPITAL)</t>
+          <t>KABUGAO</t>
         </is>
       </c>
       <c r="B49" t="n">
@@ -1943,7 +1943,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>LA TRINIDAD (CAPITAL)</t>
+          <t>LA TRINIDAD</t>
         </is>
       </c>
       <c r="B61" t="n">
@@ -2243,7 +2243,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>LAGAWE (CAPITAL)</t>
+          <t>LAGAWE</t>
         </is>
       </c>
       <c r="B73" t="n">
@@ -2468,7 +2468,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CITY OF TABUK (CAPITAL)</t>
+          <t>CITY OF TABUK</t>
         </is>
       </c>
       <c r="B82" t="n">
@@ -2618,7 +2618,7 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>BONTOC (CAPITAL)</t>
+          <t>BONTOC</t>
         </is>
       </c>
       <c r="B88" t="n">
@@ -3068,7 +3068,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>CITY OF LAOAG (CAPITAL)</t>
+          <t>CITY OF LAOAG</t>
         </is>
       </c>
       <c r="B106" t="n">
@@ -4193,7 +4193,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>CITY OF VIGAN (CAPITAL)</t>
+          <t>CITY OF VIGAN</t>
         </is>
       </c>
       <c r="B151" t="n">
@@ -4543,7 +4543,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>CITY OF SAN FERNANDO (CAPITAL)</t>
+          <t>CITY OF SAN FERNANDO</t>
         </is>
       </c>
       <c r="B165" t="n">
@@ -5268,7 +5268,7 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>LINGAYEN (CAPITAL)</t>
+          <t>LINGAYEN</t>
         </is>
       </c>
       <c r="B194" t="n">
@@ -5918,7 +5918,7 @@
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>BASCO (CAPITAL)</t>
+          <t>BASCO</t>
         </is>
       </c>
       <c r="B220" t="n">
@@ -6693,7 +6693,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>SANTO NIÑO (FAIRE)</t>
+          <t>SANTO NIÑO</t>
         </is>
       </c>
       <c r="B251" t="n">
@@ -6768,7 +6768,7 @@
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>TUGUEGARAO CITY (CAPITAL)</t>
+          <t>TUGUEGARAO CITY</t>
         </is>
       </c>
       <c r="B254" t="n">
@@ -7143,7 +7143,7 @@
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>CITY OF ILAGAN (CAPITAL)</t>
+          <t>CITY OF ILAGAN</t>
         </is>
       </c>
       <c r="B269" t="n">
@@ -7843,7 +7843,7 @@
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>BAYOMBONG (CAPITAL)</t>
+          <t>BAYOMBONG</t>
         </is>
       </c>
       <c r="B297" t="n">
@@ -8118,7 +8118,7 @@
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>CABARROGUIS (CAPITAL)</t>
+          <t>CABARROGUIS</t>
         </is>
       </c>
       <c r="B308" t="n">
@@ -8243,7 +8243,7 @@
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>BALER (CAPITAL)</t>
+          <t>BALER</t>
         </is>
       </c>
       <c r="B313" t="n">
@@ -8493,7 +8493,7 @@
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>CITY OF BALANGA (CAPITAL)</t>
+          <t>CITY OF BALANGA</t>
         </is>
       </c>
       <c r="B323" t="n">
@@ -8993,7 +8993,7 @@
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>CITY OF MALOLOS (CAPITAL)</t>
+          <t>CITY OF MALOLOS</t>
         </is>
       </c>
       <c r="B343" t="n">
@@ -9793,7 +9793,7 @@
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>CITY OF PALAYAN (CAPITAL)</t>
+          <t>CITY OF PALAYAN</t>
         </is>
       </c>
       <c r="B375" t="n">
@@ -10493,7 +10493,7 @@
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>CITY OF SAN FERNANDO (CAPITAL)</t>
+          <t>CITY OF SAN FERNANDO</t>
         </is>
       </c>
       <c r="B403" t="n">
@@ -11068,7 +11068,7 @@
     <row r="426">
       <c r="A426" t="inlineStr">
         <is>
-          <t>CITY OF TARLAC (CAPITAL)</t>
+          <t>CITY OF TARLAC</t>
         </is>
       </c>
       <c r="B426" t="n">
@@ -11218,7 +11218,7 @@
     <row r="432">
       <c r="A432" t="inlineStr">
         <is>
-          <t>IBA (CAPITAL)</t>
+          <t>IBA</t>
         </is>
       </c>
       <c r="B432" t="n">
@@ -11543,7 +11543,7 @@
     <row r="445">
       <c r="A445" t="inlineStr">
         <is>
-          <t>BATANGAS CITY (CAPITAL)</t>
+          <t>BATANGAS CITY</t>
         </is>
       </c>
       <c r="B445" t="n">
@@ -12843,7 +12843,7 @@
     <row r="497">
       <c r="A497" t="inlineStr">
         <is>
-          <t>CITY OF TRECE MARTIRES (CAPITAL)</t>
+          <t>CITY OF TRECE MARTIRES</t>
         </is>
       </c>
       <c r="B497" t="n">
@@ -13493,7 +13493,7 @@
     <row r="523">
       <c r="A523" t="inlineStr">
         <is>
-          <t>SANTA CRUZ (CAPITAL)</t>
+          <t>SANTA CRUZ</t>
         </is>
       </c>
       <c r="B523" t="n">
@@ -14643,7 +14643,7 @@
     <row r="569">
       <c r="A569" t="inlineStr">
         <is>
-          <t>CITY OF ANTIPOLO (CAPITAL)</t>
+          <t>CITY OF ANTIPOLO</t>
         </is>
       </c>
       <c r="B569" t="n">
@@ -14968,7 +14968,7 @@
     <row r="582">
       <c r="A582" t="inlineStr">
         <is>
-          <t>BOAC (CAPITAL)</t>
+          <t>BOAC</t>
         </is>
       </c>
       <c r="B582" t="n">
@@ -15243,7 +15243,7 @@
     <row r="593">
       <c r="A593" t="inlineStr">
         <is>
-          <t>MAMBURAO (CAPITAL)</t>
+          <t>MAMBURAO</t>
         </is>
       </c>
       <c r="B593" t="n">
@@ -15493,7 +15493,7 @@
     <row r="603">
       <c r="A603" t="inlineStr">
         <is>
-          <t>CITY OF CALAPAN (CAPITAL)</t>
+          <t>CITY OF CALAPAN</t>
         </is>
       </c>
       <c r="B603" t="n">
@@ -16593,7 +16593,7 @@
     <row r="647">
       <c r="A647" t="inlineStr">
         <is>
-          <t>ROMBLON (CAPITAL)</t>
+          <t>ROMBLON</t>
         </is>
       </c>
       <c r="B647" t="n">
@@ -16893,7 +16893,7 @@
     <row r="659">
       <c r="A659" t="inlineStr">
         <is>
-          <t>CITY OF LEGAZPI (CAPITAL)</t>
+          <t>CITY OF LEGAZPI</t>
         </is>
       </c>
       <c r="B659" t="n">
@@ -17268,7 +17268,7 @@
     <row r="674">
       <c r="A674" t="inlineStr">
         <is>
-          <t>DAET (CAPITAL)</t>
+          <t>DAET</t>
         </is>
       </c>
       <c r="B674" t="n">
@@ -18193,7 +18193,7 @@
     <row r="711">
       <c r="A711" t="inlineStr">
         <is>
-          <t>PILI (CAPITAL)</t>
+          <t>PILI</t>
         </is>
       </c>
       <c r="B711" t="n">
@@ -18693,7 +18693,7 @@
     <row r="731">
       <c r="A731" t="inlineStr">
         <is>
-          <t>VIRAC (CAPITAL)</t>
+          <t>VIRAC</t>
         </is>
       </c>
       <c r="B731" t="n">
@@ -18968,7 +18968,7 @@
     <row r="742">
       <c r="A742" t="inlineStr">
         <is>
-          <t>CITY OF MASBATE (CAPITAL)</t>
+          <t>CITY OF MASBATE</t>
         </is>
       </c>
       <c r="B742" t="n">
@@ -19593,7 +19593,7 @@
     <row r="767">
       <c r="A767" t="inlineStr">
         <is>
-          <t>CITY OF SORSOGON (CAPITAL)</t>
+          <t>CITY OF SORSOGON</t>
         </is>
       </c>
       <c r="B767" t="n">
@@ -19768,7 +19768,7 @@
     <row r="774">
       <c r="A774" t="inlineStr">
         <is>
-          <t>KALIBO (CAPITAL)</t>
+          <t>KALIBO</t>
         </is>
       </c>
       <c r="B774" t="n">
@@ -20318,7 +20318,7 @@
     <row r="796">
       <c r="A796" t="inlineStr">
         <is>
-          <t>SAN JOSE (CAPITAL)</t>
+          <t>SAN JOSE</t>
         </is>
       </c>
       <c r="B796" t="n">
@@ -20818,7 +20818,7 @@
     <row r="816">
       <c r="A816" t="inlineStr">
         <is>
-          <t>CITY OF ROXAS (CAPITAL)</t>
+          <t>CITY OF ROXAS</t>
         </is>
       </c>
       <c r="B816" t="n">
@@ -20943,7 +20943,7 @@
     <row r="821">
       <c r="A821" t="inlineStr">
         <is>
-          <t>JORDAN (CAPITAL)</t>
+          <t>JORDAN</t>
         </is>
       </c>
       <c r="B821" t="n">
@@ -23943,7 +23943,7 @@
     <row r="941">
       <c r="A941" t="inlineStr">
         <is>
-          <t>CITY OF TAGBILARAN (CAPITAL)</t>
+          <t>CITY OF TAGBILARAN</t>
         </is>
       </c>
       <c r="B941" t="n">
@@ -25568,7 +25568,7 @@
     <row r="1006">
       <c r="A1006" t="inlineStr">
         <is>
-          <t>CITY OF DUMAGUETE (CAPITAL)</t>
+          <t>CITY OF DUMAGUETE</t>
         </is>
       </c>
       <c r="B1006" t="n">
@@ -26093,7 +26093,7 @@
     <row r="1027">
       <c r="A1027" t="inlineStr">
         <is>
-          <t>SIQUIJOR (CAPITAL)</t>
+          <t>SIQUIJOR</t>
         </is>
       </c>
       <c r="B1027" t="n">
@@ -26293,7 +26293,7 @@
     <row r="1035">
       <c r="A1035" t="inlineStr">
         <is>
-          <t>NAVAL (CAPITAL)</t>
+          <t>NAVAL</t>
         </is>
       </c>
       <c r="B1035" t="n">
@@ -26393,7 +26393,7 @@
     <row r="1039">
       <c r="A1039" t="inlineStr">
         <is>
-          <t>CITY OF BORONGAN (CAPITAL)</t>
+          <t>CITY OF BORONGAN</t>
         </is>
       </c>
       <c r="B1039" t="n">
@@ -28043,7 +28043,7 @@
     <row r="1105">
       <c r="A1105" t="inlineStr">
         <is>
-          <t>CATARMAN (CAPITAL)</t>
+          <t>CATARMAN</t>
         </is>
       </c>
       <c r="B1105" t="n">
@@ -28643,7 +28643,7 @@
     <row r="1129">
       <c r="A1129" t="inlineStr">
         <is>
-          <t>CITY OF CATBALOGAN (CAPITAL)</t>
+          <t>CITY OF CATBALOGAN</t>
         </is>
       </c>
       <c r="B1129" t="n">
@@ -29368,7 +29368,7 @@
     <row r="1158">
       <c r="A1158" t="inlineStr">
         <is>
-          <t>CITY OF MAASIN (CAPITAL)</t>
+          <t>CITY OF MAASIN</t>
         </is>
       </c>
       <c r="B1158" t="n">
@@ -29743,7 +29743,7 @@
     <row r="1173">
       <c r="A1173" t="inlineStr">
         <is>
-          <t>CITY OF DIPOLOG (CAPITAL)</t>
+          <t>CITY OF DIPOLOG</t>
         </is>
       </c>
       <c r="B1173" t="n">
@@ -30743,7 +30743,7 @@
     <row r="1213">
       <c r="A1213" t="inlineStr">
         <is>
-          <t>CITY OF PAGADIAN (CAPITAL)</t>
+          <t>CITY OF PAGADIAN</t>
         </is>
       </c>
       <c r="B1213" t="n">
@@ -31118,7 +31118,7 @@
     <row r="1228">
       <c r="A1228" t="inlineStr">
         <is>
-          <t>IPIL (CAPITAL)</t>
+          <t>IPIL</t>
         </is>
       </c>
       <c r="B1228" t="n">
@@ -31718,7 +31718,7 @@
     <row r="1252">
       <c r="A1252" t="inlineStr">
         <is>
-          <t>CITY OF MALAYBALAY (CAPITAL)</t>
+          <t>CITY OF MALAYBALAY</t>
         </is>
       </c>
       <c r="B1252" t="n">
@@ -32043,7 +32043,7 @@
     <row r="1265">
       <c r="A1265" t="inlineStr">
         <is>
-          <t>MAMBAJAO (CAPITAL)</t>
+          <t>MAMBAJAO</t>
         </is>
       </c>
       <c r="B1265" t="n">
@@ -32618,7 +32618,7 @@
     <row r="1288">
       <c r="A1288" t="inlineStr">
         <is>
-          <t>TUBOD (CAPITAL)</t>
+          <t>TUBOD</t>
         </is>
       </c>
       <c r="B1288" t="n">
@@ -32868,7 +32868,7 @@
     <row r="1298">
       <c r="A1298" t="inlineStr">
         <is>
-          <t>CITY OF OROQUIETA (CAPITAL)</t>
+          <t>CITY OF OROQUIETA</t>
         </is>
       </c>
       <c r="B1298" t="n">
@@ -33893,7 +33893,7 @@
     <row r="1339">
       <c r="A1339" t="inlineStr">
         <is>
-          <t>NABUNTURAN (CAPITAL)</t>
+          <t>NABUNTURAN</t>
         </is>
       </c>
       <c r="B1339" t="n">
@@ -34193,7 +34193,7 @@
     <row r="1351">
       <c r="A1351" t="inlineStr">
         <is>
-          <t>CITY OF TAGUM (CAPITAL)</t>
+          <t>CITY OF TAGUM</t>
         </is>
       </c>
       <c r="B1351" t="n">
@@ -34268,7 +34268,7 @@
     <row r="1354">
       <c r="A1354" t="inlineStr">
         <is>
-          <t>CITY OF DIGOS (CAPITAL)</t>
+          <t>CITY OF DIGOS</t>
         </is>
       </c>
       <c r="B1354" t="n">
@@ -34543,7 +34543,7 @@
     <row r="1365">
       <c r="A1365" t="inlineStr">
         <is>
-          <t>MALITA (CAPITAL)</t>
+          <t>MALITA</t>
         </is>
       </c>
       <c r="B1365" t="n">
@@ -34818,7 +34818,7 @@
     <row r="1376">
       <c r="A1376" t="inlineStr">
         <is>
-          <t>CITY OF MATI (CAPITAL)</t>
+          <t>CITY OF MATI</t>
         </is>
       </c>
       <c r="B1376" t="n">
@@ -35068,7 +35068,7 @@
     <row r="1386">
       <c r="A1386" t="inlineStr">
         <is>
-          <t>CITY OF KIDAPAWAN (CAPITAL)</t>
+          <t>CITY OF KIDAPAWAN</t>
         </is>
       </c>
       <c r="B1386" t="n">
@@ -35343,7 +35343,7 @@
     <row r="1397">
       <c r="A1397" t="inlineStr">
         <is>
-          <t>ALABEL (CAPITAL)</t>
+          <t>ALABEL</t>
         </is>
       </c>
       <c r="B1397" t="n">
@@ -35543,7 +35543,7 @@
     <row r="1405">
       <c r="A1405" t="inlineStr">
         <is>
-          <t>CITY OF KORONADAL (CAPITAL)</t>
+          <t>CITY OF KORONADAL</t>
         </is>
       </c>
       <c r="B1405" t="n">
@@ -35868,7 +35868,7 @@
     <row r="1418">
       <c r="A1418" t="inlineStr">
         <is>
-          <t>ISULAN (CAPITAL)</t>
+          <t>ISULAN</t>
         </is>
       </c>
       <c r="B1418" t="n">
@@ -36118,7 +36118,7 @@
     <row r="1428">
       <c r="A1428" t="inlineStr">
         <is>
-          <t>CITY OF CABADBARAN (CAPITAL)</t>
+          <t>CITY OF CABADBARAN</t>
         </is>
       </c>
       <c r="B1428" t="n">
@@ -36493,7 +36493,7 @@
     <row r="1443">
       <c r="A1443" t="inlineStr">
         <is>
-          <t>PROSPERIDAD (CAPITAL)</t>
+          <t>PROSPERIDAD</t>
         </is>
       </c>
       <c r="B1443" t="n">
@@ -36843,7 +36843,7 @@
     <row r="1457">
       <c r="A1457" t="inlineStr">
         <is>
-          <t>SAN JOSE (CAPITAL)</t>
+          <t>SAN JOSE</t>
         </is>
       </c>
       <c r="B1457" t="n">
@@ -37343,7 +37343,7 @@
     <row r="1477">
       <c r="A1477" t="inlineStr">
         <is>
-          <t>CITY OF SURIGAO (CAPITAL)</t>
+          <t>CITY OF SURIGAO</t>
         </is>
       </c>
       <c r="B1477" t="n">
@@ -37868,7 +37868,7 @@
     <row r="1498">
       <c r="A1498" t="inlineStr">
         <is>
-          <t>CITY OF TANDAG (CAPITAL)</t>
+          <t>CITY OF TANDAG</t>
         </is>
       </c>
       <c r="B1498" t="n">
@@ -37993,7 +37993,7 @@
     <row r="1503">
       <c r="A1503" t="inlineStr">
         <is>
-          <t>CITY OF LAMITAN (CAPITAL)</t>
+          <t>CITY OF LAMITAN</t>
         </is>
       </c>
       <c r="B1503" t="n">
@@ -38768,7 +38768,7 @@
     <row r="1534">
       <c r="A1534" t="inlineStr">
         <is>
-          <t>CITY OF MARAWI (CAPITAL)</t>
+          <t>CITY OF MARAWI</t>
         </is>
       </c>
       <c r="B1534" t="n">
@@ -39893,7 +39893,7 @@
     <row r="1579">
       <c r="A1579" t="inlineStr">
         <is>
-          <t>SHARIFF AGUAK (MAGANOY) (CAPITAL)</t>
+          <t>SHARIFF AGUAK (MAGANOY)</t>
         </is>
       </c>
       <c r="B1579" t="n">
@@ -40168,7 +40168,7 @@
     <row r="1590">
       <c r="A1590" t="inlineStr">
         <is>
-          <t>JOLO (CAPITAL)</t>
+          <t>JOLO</t>
         </is>
       </c>
       <c r="B1590" t="n">
@@ -40593,7 +40593,7 @@
     <row r="1607">
       <c r="A1607" t="inlineStr">
         <is>
-          <t>BONGAO (CAPITAL)</t>
+          <t>BONGAO</t>
         </is>
       </c>
       <c r="B1607" t="n">

</xml_diff>